<commit_message>
added hostnames and screen IDs
</commit_message>
<xml_diff>
--- a/program.xlsx
+++ b/program.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10510"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/marco/work/git/gwadw2026/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2525257-21ED-C347-9976-90BCA4FB2016}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="240" yWindow="660" windowWidth="24040" windowHeight="14060" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Conference" sheetId="1" r:id="rId1"/>
@@ -20,12 +26,12 @@
     <sheet name="48418" sheetId="11" r:id="rId11"/>
     <sheet name="48419" sheetId="12" r:id="rId12"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="326" uniqueCount="237">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="354" uniqueCount="264">
   <si>
     <t>Key</t>
   </si>
@@ -96,18 +102,6 @@
     <t>Poster Session: Others</t>
   </si>
   <si>
-    <t>2026-05-19 18:00:00</t>
-  </si>
-  <si>
-    <t>2026-05-21 18:00:00</t>
-  </si>
-  <si>
-    <t>2026-05-19 19:30:00</t>
-  </si>
-  <si>
-    <t>2026-05-21 19:30:00</t>
-  </si>
-  <si>
     <t>Hostname</t>
   </si>
   <si>
@@ -736,13 +730,106 @@
   </si>
   <si>
     <t>Stanford University</t>
+  </si>
+  <si>
+    <t>pi5pm1</t>
+  </si>
+  <si>
+    <t>pi5pm2</t>
+  </si>
+  <si>
+    <t>pi5pm3</t>
+  </si>
+  <si>
+    <t>pi5pm4</t>
+  </si>
+  <si>
+    <t>pi5pm5</t>
+  </si>
+  <si>
+    <t>pi5pm6</t>
+  </si>
+  <si>
+    <t>pi5pm7</t>
+  </si>
+  <si>
+    <t>pi5pm8</t>
+  </si>
+  <si>
+    <t>pi5pm9</t>
+  </si>
+  <si>
+    <t>pi5pm10</t>
+  </si>
+  <si>
+    <t>pi5pm11</t>
+  </si>
+  <si>
+    <t>pi5pm12</t>
+  </si>
+  <si>
+    <t>pi5pm13</t>
+  </si>
+  <si>
+    <t>pi5pm14</t>
+  </si>
+  <si>
+    <t>pi5pm15</t>
+  </si>
+  <si>
+    <t>pi5pm16</t>
+  </si>
+  <si>
+    <t>pi5pm17</t>
+  </si>
+  <si>
+    <t>pi5pm18</t>
+  </si>
+  <si>
+    <t>pi5pm19</t>
+  </si>
+  <si>
+    <t>pi5pm20</t>
+  </si>
+  <si>
+    <t>pi5pm21</t>
+  </si>
+  <si>
+    <t>pi5pm22</t>
+  </si>
+  <si>
+    <t>pi5pm23</t>
+  </si>
+  <si>
+    <t>pi5pm24</t>
+  </si>
+  <si>
+    <t>pi5pm25</t>
+  </si>
+  <si>
+    <t>pi5pm26</t>
+  </si>
+  <si>
+    <t>pi5pm27</t>
+  </si>
+  <si>
+    <t>pi5pm28</t>
+  </si>
+  <si>
+    <t>2025-05-19 18:00:00</t>
+  </si>
+  <si>
+    <t>2026-05-20 21:00:00</t>
+  </si>
+  <si>
+    <t>2026-05-22 19:30:00</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -771,21 +858,30 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normale" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -823,7 +919,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -857,6 +953,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -891,9 +988,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1066,15 +1164,15 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B5"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="25.7109375" customWidth="1"/>
-    <col min="2" max="2" width="100.7109375" customWidth="1"/>
+    <col min="1" max="1" width="25.6640625" customWidth="1"/>
+    <col min="2" max="2" width="100.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1082,7 +1180,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -1090,7 +1188,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:2">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -1098,7 +1196,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:2">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -1106,7 +1204,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:2">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>5</v>
       </c>
@@ -1120,85 +1218,94 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
   <dimension ref="A1:F4"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="2" width="12.7109375" customWidth="1"/>
-    <col min="3" max="3" width="100.7109375" customWidth="1"/>
-    <col min="4" max="5" width="20.7109375" customWidth="1"/>
-    <col min="6" max="6" width="60.7109375" customWidth="1"/>
+    <col min="1" max="2" width="12.6640625" customWidth="1"/>
+    <col min="3" max="3" width="100.6640625" customWidth="1"/>
+    <col min="4" max="5" width="20.6640625" customWidth="1"/>
+    <col min="6" max="6" width="60.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D1" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" t="s">
+        <v>28</v>
+      </c>
+      <c r="F1" t="s">
         <v>29</v>
       </c>
-      <c r="B1" t="s">
-        <v>28</v>
-      </c>
-      <c r="C1" t="s">
-        <v>30</v>
-      </c>
-      <c r="D1" t="s">
-        <v>31</v>
-      </c>
-      <c r="E1" t="s">
-        <v>32</v>
-      </c>
-      <c r="F1" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6">
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>56</v>
       </c>
+      <c r="B2">
+        <v>20</v>
+      </c>
       <c r="C2" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
       <c r="D2" t="s">
-        <v>209</v>
+        <v>205</v>
       </c>
       <c r="E2" t="s">
-        <v>212</v>
+        <v>208</v>
       </c>
       <c r="F2" t="s">
-        <v>215</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>66</v>
       </c>
+      <c r="B3">
+        <v>21</v>
+      </c>
       <c r="C3" t="s">
-        <v>207</v>
+        <v>203</v>
       </c>
       <c r="D3" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="E3" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="F3" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>80</v>
       </c>
+      <c r="B4">
+        <v>22</v>
+      </c>
       <c r="C4" t="s">
-        <v>208</v>
+        <v>204</v>
       </c>
       <c r="D4" t="s">
-        <v>211</v>
+        <v>207</v>
       </c>
       <c r="E4" t="s">
-        <v>214</v>
+        <v>210</v>
       </c>
       <c r="F4" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
     </row>
   </sheetData>
@@ -1207,102 +1314,114 @@
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
   <dimension ref="A1:F5"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="2" width="12.7109375" customWidth="1"/>
-    <col min="3" max="3" width="100.7109375" customWidth="1"/>
-    <col min="4" max="5" width="20.7109375" customWidth="1"/>
-    <col min="6" max="6" width="60.7109375" customWidth="1"/>
+    <col min="1" max="2" width="12.6640625" customWidth="1"/>
+    <col min="3" max="3" width="100.6640625" customWidth="1"/>
+    <col min="4" max="5" width="20.6640625" customWidth="1"/>
+    <col min="6" max="6" width="60.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D1" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" t="s">
+        <v>28</v>
+      </c>
+      <c r="F1" t="s">
         <v>29</v>
       </c>
-      <c r="B1" t="s">
-        <v>28</v>
-      </c>
-      <c r="C1" t="s">
-        <v>30</v>
-      </c>
-      <c r="D1" t="s">
-        <v>31</v>
-      </c>
-      <c r="E1" t="s">
-        <v>32</v>
-      </c>
-      <c r="F1" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6">
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>1</v>
       </c>
+      <c r="B2">
+        <v>23</v>
+      </c>
       <c r="C2" t="s">
+        <v>214</v>
+      </c>
+      <c r="D2" t="s">
         <v>218</v>
       </c>
-      <c r="D2" t="s">
-        <v>222</v>
-      </c>
       <c r="E2" t="s">
+        <v>221</v>
+      </c>
+      <c r="F2" t="s">
         <v>225</v>
       </c>
-      <c r="F2" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6">
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>69</v>
       </c>
+      <c r="B3">
+        <v>24</v>
+      </c>
       <c r="C3" t="s">
-        <v>219</v>
+        <v>215</v>
       </c>
       <c r="D3" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="E3" t="s">
+        <v>222</v>
+      </c>
+      <c r="F3" t="s">
         <v>226</v>
       </c>
-      <c r="F3" t="s">
-        <v>230</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6">
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>90</v>
       </c>
+      <c r="B4">
+        <v>25</v>
+      </c>
       <c r="C4" t="s">
-        <v>220</v>
+        <v>216</v>
       </c>
       <c r="D4" t="s">
+        <v>219</v>
+      </c>
+      <c r="E4" t="s">
         <v>223</v>
       </c>
-      <c r="E4" t="s">
-        <v>227</v>
-      </c>
       <c r="F4" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>119</v>
       </c>
+      <c r="B5">
+        <v>26</v>
+      </c>
       <c r="C5" t="s">
-        <v>221</v>
+        <v>217</v>
       </c>
       <c r="D5" t="s">
+        <v>220</v>
+      </c>
+      <c r="E5" t="s">
         <v>224</v>
       </c>
-      <c r="E5" t="s">
-        <v>228</v>
-      </c>
       <c r="F5" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
     </row>
   </sheetData>
@@ -1311,65 +1430,71 @@
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
   <dimension ref="A1:F3"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="2" width="12.7109375" customWidth="1"/>
-    <col min="3" max="3" width="100.7109375" customWidth="1"/>
-    <col min="4" max="5" width="20.7109375" customWidth="1"/>
-    <col min="6" max="6" width="60.7109375" customWidth="1"/>
+    <col min="1" max="2" width="12.6640625" customWidth="1"/>
+    <col min="3" max="3" width="100.6640625" customWidth="1"/>
+    <col min="4" max="5" width="20.6640625" customWidth="1"/>
+    <col min="6" max="6" width="60.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D1" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" t="s">
+        <v>28</v>
+      </c>
+      <c r="F1" t="s">
         <v>29</v>
       </c>
-      <c r="B1" t="s">
-        <v>28</v>
-      </c>
-      <c r="C1" t="s">
-        <v>30</v>
-      </c>
-      <c r="D1" t="s">
-        <v>31</v>
-      </c>
-      <c r="E1" t="s">
-        <v>32</v>
-      </c>
-      <c r="F1" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6">
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>3</v>
       </c>
+      <c r="B2">
+        <v>27</v>
+      </c>
       <c r="C2" t="s">
-        <v>231</v>
+        <v>227</v>
       </c>
       <c r="D2" t="s">
-        <v>233</v>
+        <v>229</v>
       </c>
       <c r="E2" t="s">
-        <v>234</v>
+        <v>230</v>
       </c>
       <c r="F2" t="s">
-        <v>236</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>11</v>
       </c>
+      <c r="B3">
+        <v>28</v>
+      </c>
       <c r="C3" t="s">
-        <v>232</v>
+        <v>228</v>
       </c>
       <c r="D3" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="E3" t="s">
-        <v>235</v>
+        <v>231</v>
       </c>
     </row>
   </sheetData>
@@ -1378,16 +1503,16 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:D10"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="12.7109375" customWidth="1"/>
-    <col min="2" max="2" width="100.7109375" customWidth="1"/>
-    <col min="3" max="4" width="20.7109375" customWidth="1"/>
+    <col min="1" max="1" width="12.6640625" customWidth="1"/>
+    <col min="2" max="2" width="100.6640625" customWidth="1"/>
+    <col min="3" max="4" width="20.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>10</v>
       </c>
@@ -1401,130 +1526,130 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:4">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>48411</v>
       </c>
       <c r="B2" t="s">
         <v>14</v>
       </c>
-      <c r="C2" t="s">
-        <v>23</v>
-      </c>
-      <c r="D2" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4">
+      <c r="C2" s="1" t="s">
+        <v>261</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>48412</v>
       </c>
       <c r="B3" t="s">
         <v>15</v>
       </c>
-      <c r="C3" t="s">
-        <v>23</v>
-      </c>
-      <c r="D3" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4">
+      <c r="C3" s="1" t="s">
+        <v>261</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>48413</v>
       </c>
       <c r="B4" t="s">
         <v>16</v>
       </c>
-      <c r="C4" t="s">
-        <v>23</v>
-      </c>
-      <c r="D4" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4">
+      <c r="C4" s="1" t="s">
+        <v>261</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>48414</v>
       </c>
       <c r="B5" t="s">
         <v>17</v>
       </c>
-      <c r="C5" t="s">
-        <v>23</v>
-      </c>
-      <c r="D5" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4">
+      <c r="C5" s="1" t="s">
+        <v>261</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>48415</v>
       </c>
       <c r="B6" t="s">
         <v>18</v>
       </c>
-      <c r="C6" t="s">
-        <v>24</v>
-      </c>
-      <c r="D6" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4">
+      <c r="C6" s="1" t="s">
+        <v>262</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>48416</v>
       </c>
       <c r="B7" t="s">
         <v>19</v>
       </c>
-      <c r="C7" t="s">
-        <v>24</v>
-      </c>
-      <c r="D7" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4">
+      <c r="C7" s="1" t="s">
+        <v>262</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>48417</v>
       </c>
       <c r="B8" t="s">
         <v>20</v>
       </c>
-      <c r="C8" t="s">
-        <v>24</v>
-      </c>
-      <c r="D8" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4">
+      <c r="C8" s="1" t="s">
+        <v>262</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>48418</v>
       </c>
       <c r="B9" t="s">
         <v>21</v>
       </c>
-      <c r="C9" t="s">
-        <v>24</v>
-      </c>
-      <c r="D9" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4">
+      <c r="C9" s="1" t="s">
+        <v>262</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>48419</v>
       </c>
       <c r="B10" t="s">
         <v>22</v>
       </c>
-      <c r="C10" t="s">
-        <v>24</v>
-      </c>
-      <c r="D10" t="s">
-        <v>26</v>
+      <c r="C10" s="1" t="s">
+        <v>262</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>263</v>
       </c>
     </row>
   </sheetData>
@@ -1533,18 +1658,242 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B1"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <dimension ref="A1:B29"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="2" width="20.7109375" customWidth="1"/>
+    <col min="1" max="2" width="20.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>233</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>234</v>
+      </c>
+      <c r="B3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>235</v>
+      </c>
+      <c r="B4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>236</v>
+      </c>
+      <c r="B5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>237</v>
+      </c>
+      <c r="B6">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>238</v>
+      </c>
+      <c r="B7">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>239</v>
+      </c>
+      <c r="B8">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>240</v>
+      </c>
+      <c r="B9">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>241</v>
+      </c>
+      <c r="B10">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>242</v>
+      </c>
+      <c r="B11">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>243</v>
+      </c>
+      <c r="B12">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>244</v>
+      </c>
+      <c r="B13">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>245</v>
+      </c>
+      <c r="B14">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>246</v>
+      </c>
+      <c r="B15">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>247</v>
+      </c>
+      <c r="B16">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>248</v>
+      </c>
+      <c r="B17">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>249</v>
+      </c>
+      <c r="B18">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>250</v>
+      </c>
+      <c r="B19">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>251</v>
+      </c>
+      <c r="B20">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>252</v>
+      </c>
+      <c r="B21">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>253</v>
+      </c>
+      <c r="B22">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
+        <v>254</v>
+      </c>
+      <c r="B23">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A24" t="s">
+        <v>255</v>
+      </c>
+      <c r="B24">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A25" t="s">
+        <v>256</v>
+      </c>
+      <c r="B25">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A26" t="s">
+        <v>257</v>
+      </c>
+      <c r="B26">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A27" t="s">
+        <v>258</v>
+      </c>
+      <c r="B27">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A28" t="s">
+        <v>259</v>
+      </c>
+      <c r="B28">
         <v>27</v>
       </c>
-      <c r="B1" t="s">
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A29" t="s">
+        <v>260</v>
+      </c>
+      <c r="B29">
         <v>28</v>
       </c>
     </row>
@@ -1554,255 +1903,294 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:F14"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="2" width="12.7109375" customWidth="1"/>
-    <col min="3" max="3" width="100.7109375" customWidth="1"/>
-    <col min="4" max="5" width="20.7109375" customWidth="1"/>
-    <col min="6" max="6" width="60.7109375" customWidth="1"/>
+    <col min="1" max="2" width="12.6640625" customWidth="1"/>
+    <col min="3" max="3" width="100.6640625" customWidth="1"/>
+    <col min="4" max="5" width="20.6640625" customWidth="1"/>
+    <col min="6" max="6" width="60.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D1" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" t="s">
+        <v>28</v>
+      </c>
+      <c r="F1" t="s">
         <v>29</v>
       </c>
-      <c r="B1" t="s">
-        <v>28</v>
-      </c>
-      <c r="C1" t="s">
-        <v>30</v>
-      </c>
-      <c r="D1" t="s">
-        <v>31</v>
-      </c>
-      <c r="E1" t="s">
-        <v>32</v>
-      </c>
-      <c r="F1" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6">
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>19</v>
       </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
       <c r="C2" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="D2" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="E2" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="F2" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>27</v>
       </c>
+      <c r="B3">
+        <v>2</v>
+      </c>
       <c r="C3" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="D3" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="E3" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="F3" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>32</v>
       </c>
+      <c r="B4">
+        <v>3</v>
+      </c>
       <c r="C4" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="D4" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="E4" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="F4" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>42</v>
       </c>
+      <c r="B5">
+        <v>4</v>
+      </c>
       <c r="C5" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="D5" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="E5" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="F5" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>44</v>
       </c>
+      <c r="B6">
+        <v>5</v>
+      </c>
       <c r="C6" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="D6" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="E6" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="F6" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>70</v>
       </c>
+      <c r="B7">
+        <v>6</v>
+      </c>
       <c r="C7" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="D7" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="E7" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="F7" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>76</v>
       </c>
+      <c r="B8">
+        <v>7</v>
+      </c>
       <c r="C8" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="D8" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="E8" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="F8" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>78</v>
       </c>
+      <c r="B9">
+        <v>8</v>
+      </c>
       <c r="C9" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="D9" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="E9" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="F9" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>84</v>
       </c>
+      <c r="B10">
+        <v>9</v>
+      </c>
       <c r="C10" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="D10" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="E10" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="F10" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>92</v>
       </c>
+      <c r="B11">
+        <v>10</v>
+      </c>
       <c r="C11" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="D11" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="E11" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="F11" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>103</v>
       </c>
+      <c r="B12">
+        <v>11</v>
+      </c>
       <c r="C12" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="D12" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="E12" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="F12" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>122</v>
       </c>
+      <c r="B13">
+        <v>12</v>
+      </c>
       <c r="C13" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="D13" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="E13" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="F13" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>127</v>
       </c>
+      <c r="B14">
+        <v>12</v>
+      </c>
       <c r="C14" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="D14" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="E14" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="F14" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
     </row>
   </sheetData>
@@ -1811,181 +2199,208 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:F10"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="2" width="12.7109375" customWidth="1"/>
-    <col min="3" max="3" width="100.7109375" customWidth="1"/>
-    <col min="4" max="5" width="20.7109375" customWidth="1"/>
-    <col min="6" max="6" width="60.7109375" customWidth="1"/>
+    <col min="1" max="2" width="12.6640625" customWidth="1"/>
+    <col min="3" max="3" width="100.6640625" customWidth="1"/>
+    <col min="4" max="5" width="20.6640625" customWidth="1"/>
+    <col min="6" max="6" width="60.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D1" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" t="s">
+        <v>28</v>
+      </c>
+      <c r="F1" t="s">
         <v>29</v>
       </c>
-      <c r="B1" t="s">
-        <v>28</v>
-      </c>
-      <c r="C1" t="s">
-        <v>30</v>
-      </c>
-      <c r="D1" t="s">
-        <v>31</v>
-      </c>
-      <c r="E1" t="s">
-        <v>32</v>
-      </c>
-      <c r="F1" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6">
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>17</v>
       </c>
+      <c r="B2">
+        <v>13</v>
+      </c>
       <c r="C2" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="D2" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="E2" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="F2" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>25</v>
       </c>
+      <c r="B3">
+        <v>14</v>
+      </c>
       <c r="C3" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="D3" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="E3" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="F3" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>54</v>
       </c>
+      <c r="B4">
+        <v>15</v>
+      </c>
       <c r="C4" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="D4" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="E4" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="F4" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>59</v>
       </c>
+      <c r="B5">
+        <v>16</v>
+      </c>
       <c r="C5" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="D5" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="E5" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="F5" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>60</v>
       </c>
+      <c r="B6">
+        <v>17</v>
+      </c>
       <c r="C6" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="D6" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="E6" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="F6" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>71</v>
       </c>
+      <c r="B7">
+        <v>18</v>
+      </c>
       <c r="C7" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="D7" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="E7" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>101</v>
       </c>
+      <c r="B8">
+        <v>19</v>
+      </c>
       <c r="C8" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="D8" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="E8" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>126</v>
       </c>
+      <c r="B9">
+        <v>20</v>
+      </c>
       <c r="C9" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="D9" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="E9" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="F9" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>132</v>
       </c>
+      <c r="B10">
+        <v>20</v>
+      </c>
       <c r="C10" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="D10" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="E10" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="F10" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
     </row>
   </sheetData>
@@ -1994,119 +2409,134 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:F6"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="2" width="12.7109375" customWidth="1"/>
-    <col min="3" max="3" width="100.7109375" customWidth="1"/>
-    <col min="4" max="5" width="20.7109375" customWidth="1"/>
-    <col min="6" max="6" width="60.7109375" customWidth="1"/>
+    <col min="1" max="2" width="12.6640625" customWidth="1"/>
+    <col min="3" max="3" width="100.6640625" customWidth="1"/>
+    <col min="4" max="5" width="20.6640625" customWidth="1"/>
+    <col min="6" max="6" width="60.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D1" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" t="s">
+        <v>28</v>
+      </c>
+      <c r="F1" t="s">
         <v>29</v>
       </c>
-      <c r="B1" t="s">
-        <v>28</v>
-      </c>
-      <c r="C1" t="s">
-        <v>30</v>
-      </c>
-      <c r="D1" t="s">
-        <v>31</v>
-      </c>
-      <c r="E1" t="s">
-        <v>32</v>
-      </c>
-      <c r="F1" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6">
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>13</v>
       </c>
+      <c r="B2">
+        <v>21</v>
+      </c>
       <c r="C2" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="D2" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="E2" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="F2" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>21</v>
       </c>
+      <c r="B3">
+        <v>22</v>
+      </c>
       <c r="C3" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="D3" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="E3" t="s">
+        <v>122</v>
+      </c>
+      <c r="F3" t="s">
         <v>126</v>
       </c>
-      <c r="F3" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6">
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>48</v>
       </c>
+      <c r="B4">
+        <v>23</v>
+      </c>
       <c r="C4" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="D4" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="E4" t="s">
+        <v>123</v>
+      </c>
+      <c r="F4" t="s">
         <v>127</v>
       </c>
-      <c r="F4" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6">
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>107</v>
       </c>
+      <c r="B5">
+        <v>24</v>
+      </c>
       <c r="C5" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="D5" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="E5" t="s">
+        <v>124</v>
+      </c>
+      <c r="F5" t="s">
         <v>128</v>
       </c>
-      <c r="F5" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6">
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>114</v>
       </c>
+      <c r="B6">
+        <v>25</v>
+      </c>
       <c r="C6" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="D6" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="E6" t="s">
+        <v>125</v>
+      </c>
+      <c r="F6" t="s">
         <v>129</v>
-      </c>
-      <c r="F6" t="s">
-        <v>133</v>
       </c>
     </row>
   </sheetData>
@@ -2115,85 +2545,94 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:F4"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="2" width="12.7109375" customWidth="1"/>
-    <col min="3" max="3" width="100.7109375" customWidth="1"/>
-    <col min="4" max="5" width="20.7109375" customWidth="1"/>
-    <col min="6" max="6" width="60.7109375" customWidth="1"/>
+    <col min="1" max="2" width="12.6640625" customWidth="1"/>
+    <col min="3" max="3" width="100.6640625" customWidth="1"/>
+    <col min="4" max="5" width="20.6640625" customWidth="1"/>
+    <col min="6" max="6" width="60.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D1" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" t="s">
+        <v>28</v>
+      </c>
+      <c r="F1" t="s">
         <v>29</v>
       </c>
-      <c r="B1" t="s">
-        <v>28</v>
-      </c>
-      <c r="C1" t="s">
-        <v>30</v>
-      </c>
-      <c r="D1" t="s">
-        <v>31</v>
-      </c>
-      <c r="E1" t="s">
-        <v>32</v>
-      </c>
-      <c r="F1" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6">
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>49</v>
       </c>
+      <c r="B2">
+        <v>26</v>
+      </c>
       <c r="C2" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="D2" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="E2" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="F2" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>52</v>
       </c>
+      <c r="B3">
+        <v>27</v>
+      </c>
       <c r="C3" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="D3" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="E3" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="F3" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>64</v>
       </c>
+      <c r="B4">
+        <v>28</v>
+      </c>
       <c r="C4" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="D4" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="E4" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="F4" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
     </row>
   </sheetData>
@@ -2202,186 +2641,216 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:F11"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="2" width="12.7109375" customWidth="1"/>
-    <col min="3" max="3" width="100.7109375" customWidth="1"/>
-    <col min="4" max="5" width="20.7109375" customWidth="1"/>
-    <col min="6" max="6" width="60.7109375" customWidth="1"/>
+    <col min="1" max="2" width="12.6640625" customWidth="1"/>
+    <col min="3" max="3" width="100.6640625" customWidth="1"/>
+    <col min="4" max="5" width="20.6640625" customWidth="1"/>
+    <col min="6" max="6" width="60.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D1" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" t="s">
+        <v>28</v>
+      </c>
+      <c r="F1" t="s">
         <v>29</v>
       </c>
-      <c r="B1" t="s">
-        <v>28</v>
-      </c>
-      <c r="C1" t="s">
-        <v>30</v>
-      </c>
-      <c r="D1" t="s">
-        <v>31</v>
-      </c>
-      <c r="E1" t="s">
-        <v>32</v>
-      </c>
-      <c r="F1" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6">
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>14</v>
       </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
       <c r="C2" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="D2" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="E2" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>58</v>
       </c>
+      <c r="B3">
+        <v>2</v>
+      </c>
       <c r="C3" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="D3" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="E3" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="F3" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>91</v>
       </c>
+      <c r="B4">
+        <v>3</v>
+      </c>
       <c r="C4" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="D4" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="E4" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="F4" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>93</v>
       </c>
+      <c r="B5">
+        <v>4</v>
+      </c>
       <c r="C5" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="D5" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="E5" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>94</v>
       </c>
+      <c r="B6">
+        <v>5</v>
+      </c>
       <c r="C6" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="D6" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="E6" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>95</v>
       </c>
+      <c r="B7">
+        <v>6</v>
+      </c>
       <c r="C7" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="D7" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="E7" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>97</v>
       </c>
+      <c r="B8">
+        <v>7</v>
+      </c>
       <c r="C8" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="D8" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="E8" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>99</v>
       </c>
+      <c r="B9">
+        <v>8</v>
+      </c>
       <c r="C9" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="D9" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="E9" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>104</v>
       </c>
+      <c r="B10">
+        <v>9</v>
+      </c>
       <c r="C10" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="D10" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="E10" t="s">
+        <v>161</v>
+      </c>
+      <c r="F10" t="s">
         <v>165</v>
       </c>
-      <c r="F10" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6">
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>118</v>
       </c>
+      <c r="B11">
+        <v>9</v>
+      </c>
       <c r="C11" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="D11" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="E11" t="s">
+        <v>162</v>
+      </c>
+      <c r="F11" t="s">
         <v>166</v>
-      </c>
-      <c r="F11" t="s">
-        <v>170</v>
       </c>
     </row>
   </sheetData>
@@ -2390,215 +2859,248 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
   <dimension ref="A1:F12"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="2" width="12.7109375" customWidth="1"/>
-    <col min="3" max="3" width="100.7109375" customWidth="1"/>
-    <col min="4" max="5" width="20.7109375" customWidth="1"/>
-    <col min="6" max="6" width="60.7109375" customWidth="1"/>
+    <col min="1" max="2" width="12.6640625" customWidth="1"/>
+    <col min="3" max="3" width="100.6640625" customWidth="1"/>
+    <col min="4" max="5" width="20.6640625" customWidth="1"/>
+    <col min="6" max="6" width="60.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D1" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" t="s">
+        <v>28</v>
+      </c>
+      <c r="F1" t="s">
         <v>29</v>
       </c>
-      <c r="B1" t="s">
-        <v>28</v>
-      </c>
-      <c r="C1" t="s">
-        <v>30</v>
-      </c>
-      <c r="D1" t="s">
-        <v>31</v>
-      </c>
-      <c r="E1" t="s">
-        <v>32</v>
-      </c>
-      <c r="F1" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6">
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>30</v>
       </c>
+      <c r="B2">
+        <v>10</v>
+      </c>
       <c r="C2" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="D2" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="E2" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="F2" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>46</v>
       </c>
+      <c r="B3">
+        <v>11</v>
+      </c>
       <c r="C3" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="D3" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="E3" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="F3" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>62</v>
       </c>
+      <c r="B4">
+        <v>12</v>
+      </c>
       <c r="C4" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="D4" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
       <c r="E4" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="F4" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>73</v>
       </c>
+      <c r="B5">
+        <v>13</v>
+      </c>
       <c r="C5" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="D5" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="E5" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="F5" t="s">
-        <v>201</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>75</v>
       </c>
+      <c r="B6">
+        <v>14</v>
+      </c>
       <c r="C6" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="D6" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="E6" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="F6" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>83</v>
       </c>
+      <c r="B7">
+        <v>15</v>
+      </c>
       <c r="C7" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="D7" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="E7" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="F7" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>96</v>
       </c>
+      <c r="B8">
+        <v>16</v>
+      </c>
       <c r="C8" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D8" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="E8" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>105</v>
       </c>
+      <c r="B9">
+        <v>17</v>
+      </c>
       <c r="C9" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D9" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="E9" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="F9" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>108</v>
       </c>
+      <c r="B10">
+        <v>18</v>
+      </c>
       <c r="C10" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="D10" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="E10" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>120</v>
       </c>
+      <c r="B11">
+        <v>19</v>
+      </c>
       <c r="C11" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="D11" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="E11" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
       <c r="F11" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>136</v>
       </c>
+      <c r="B12">
+        <v>19</v>
+      </c>
       <c r="C12" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="D12" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="E12" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="F12" t="s">
-        <v>205</v>
+        <v>201</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
small change to program screen ordere
</commit_message>
<xml_diff>
--- a/program.xlsx
+++ b/program.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10503"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10211"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/galli/Documents/OrgConferenze/Poster/gwadw2026/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/razzano/VirgoWork/gwadw2026/gwadw2026/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCCBACDC-A06B-5943-AC5E-578B6063F49C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D8DB173-CB8C-9240-B12D-D7BDA65D0A8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="660" windowWidth="24040" windowHeight="14060" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -875,7 +875,7 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normale" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -1973,7 +1973,7 @@
         <v>27</v>
       </c>
       <c r="B3">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="C3" t="s">
         <v>29</v>
@@ -2053,7 +2053,7 @@
         <v>70</v>
       </c>
       <c r="B7">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="C7" t="s">
         <v>33</v>
@@ -2132,9 +2132,6 @@
       <c r="A11">
         <v>92</v>
       </c>
-      <c r="B11">
-        <v>10</v>
-      </c>
       <c r="C11" t="s">
         <v>37</v>
       </c>
@@ -2153,7 +2150,7 @@
         <v>103</v>
       </c>
       <c r="B12">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C12" t="s">
         <v>38</v>
@@ -2173,7 +2170,7 @@
         <v>122</v>
       </c>
       <c r="B13">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C13" t="s">
         <v>39</v>
@@ -2193,7 +2190,7 @@
         <v>127</v>
       </c>
       <c r="B14">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="C14" t="s">
         <v>40</v>

</xml_diff>

<commit_message>
small change to program screen ordedr: removed 66
</commit_message>
<xml_diff>
--- a/program.xlsx
+++ b/program.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/razzano/VirgoWork/gwadw2026/gwadw2026/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D8DB173-CB8C-9240-B12D-D7BDA65D0A8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31EA1068-DAB4-874D-8684-4610C5B71511}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="660" windowWidth="24040" windowHeight="14060" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="660" windowWidth="24040" windowHeight="14060" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Conference" sheetId="1" r:id="rId1"/>
@@ -1284,9 +1284,6 @@
       <c r="A3">
         <v>66</v>
       </c>
-      <c r="B3">
-        <v>21</v>
-      </c>
       <c r="C3" t="s">
         <v>200</v>
       </c>
@@ -1305,7 +1302,7 @@
         <v>80</v>
       </c>
       <c r="B4">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C4" t="s">
         <v>201</v>

</xml_diff>

<commit_message>
switched posters from tue to thu
</commit_message>
<xml_diff>
--- a/program.xlsx
+++ b/program.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/razzano/VirgoWork/gwadw2026/gwadw2026/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64B0FF04-349B-4349-8EB4-78BBE73B3114}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6232DE0A-300F-3E4E-8769-B448CD8B5303}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="660" windowWidth="24040" windowHeight="14060" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="660" windowWidth="24040" windowHeight="14060" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Conference" sheetId="1" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="357" uniqueCount="260">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="349" uniqueCount="253">
   <si>
     <t>Key</t>
   </si>
@@ -456,9 +456,6 @@
     <t>Deep--Frequency Modulation Interferometry for local displacement measurements</t>
   </si>
   <si>
-    <t>Improving low frequency sensitivity for 3rd generation gravitational waves detectors</t>
-  </si>
-  <si>
     <t>Preeti</t>
   </si>
   <si>
@@ -471,9 +468,6 @@
     <t>Riccardo</t>
   </si>
   <si>
-    <t>Maria Antonietta</t>
-  </si>
-  <si>
     <t>Sharma</t>
   </si>
   <si>
@@ -486,9 +480,6 @@
     <t>Eckhardt</t>
   </si>
   <si>
-    <t>Palaia</t>
-  </si>
-  <si>
     <t>Nikhef/Maastricht University</t>
   </si>
   <si>
@@ -498,9 +489,6 @@
     <t>University of Hamburg</t>
   </si>
   <si>
-    <t>Università di Pisa and INFN-Pisa</t>
-  </si>
-  <si>
     <t>GraviTerm - A New Concept in Direct Mirror Thermal-noise Measurement</t>
   </si>
   <si>
@@ -651,18 +639,12 @@
     <t>Preliminary noise budget of a kilometric laser interferometric strainmeter for lunar geophysics and gravitational-wave astronomy</t>
   </si>
   <si>
-    <t>The Pendulum-Inverted Pendulum: simulation-driven characterization of a novel seismic isolation filter for third-generation gravitational-wave observatories</t>
-  </si>
-  <si>
     <t>James</t>
   </si>
   <si>
     <t>Léon</t>
   </si>
   <si>
-    <t>Michele</t>
-  </si>
-  <si>
     <t>Gardner</t>
   </si>
   <si>
@@ -670,9 +652,6 @@
   </si>
   <si>
     <t>Vidal</t>
-  </si>
-  <si>
-    <t>Vacatello</t>
   </si>
   <si>
     <t>University of Chicago</t>
@@ -1173,7 +1152,7 @@
         <v>2</v>
       </c>
       <c r="B2" t="s">
-        <v>251</v>
+        <v>244</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
@@ -1181,7 +1160,7 @@
         <v>3</v>
       </c>
       <c r="B3" t="s">
-        <v>250</v>
+        <v>243</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
@@ -1244,16 +1223,16 @@
         <v>20</v>
       </c>
       <c r="C2" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="D2" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="E2" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="F2" t="s">
-        <v>200</v>
+        <v>196</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
@@ -1261,16 +1240,16 @@
         <v>66</v>
       </c>
       <c r="C3" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="D3" t="s">
-        <v>195</v>
+        <v>191</v>
       </c>
       <c r="E3" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
       <c r="F3" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
@@ -1281,16 +1260,16 @@
         <v>21</v>
       </c>
       <c r="C4" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="D4" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
       <c r="E4" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="F4" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
     </row>
   </sheetData>
@@ -1334,19 +1313,19 @@
         <v>1</v>
       </c>
       <c r="B2">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C2" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="D2" t="s">
+        <v>202</v>
+      </c>
+      <c r="E2" t="s">
+        <v>204</v>
+      </c>
+      <c r="F2" t="s">
         <v>207</v>
-      </c>
-      <c r="E2" t="s">
-        <v>210</v>
-      </c>
-      <c r="F2" t="s">
-        <v>214</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
@@ -1354,19 +1333,19 @@
         <v>69</v>
       </c>
       <c r="B3">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C3" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="D3" t="s">
         <v>127</v>
       </c>
       <c r="E3" t="s">
-        <v>211</v>
+        <v>205</v>
       </c>
       <c r="F3" t="s">
-        <v>215</v>
+        <v>208</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
@@ -1374,16 +1353,16 @@
         <v>90</v>
       </c>
       <c r="B4">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C4" t="s">
-        <v>205</v>
+        <v>201</v>
       </c>
       <c r="D4" t="s">
-        <v>208</v>
+        <v>203</v>
       </c>
       <c r="E4" t="s">
-        <v>212</v>
+        <v>206</v>
       </c>
       <c r="F4" t="s">
         <v>104</v>
@@ -1391,22 +1370,22 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5">
-        <v>119</v>
+        <v>70</v>
       </c>
       <c r="B5">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C5" t="s">
-        <v>206</v>
+        <v>33</v>
       </c>
       <c r="D5" t="s">
-        <v>209</v>
+        <v>40</v>
       </c>
       <c r="E5" t="s">
-        <v>213</v>
+        <v>51</v>
       </c>
       <c r="F5" t="s">
-        <v>189</v>
+        <v>62</v>
       </c>
     </row>
   </sheetData>
@@ -1450,19 +1429,19 @@
         <v>3</v>
       </c>
       <c r="B2">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C2" t="s">
-        <v>216</v>
+        <v>209</v>
       </c>
       <c r="D2" t="s">
-        <v>218</v>
+        <v>211</v>
       </c>
       <c r="E2" t="s">
-        <v>219</v>
+        <v>212</v>
       </c>
       <c r="F2" t="s">
-        <v>221</v>
+        <v>214</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
@@ -1470,16 +1449,16 @@
         <v>11</v>
       </c>
       <c r="B3">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C3" t="s">
-        <v>217</v>
+        <v>210</v>
       </c>
       <c r="D3" t="s">
         <v>45</v>
       </c>
       <c r="E3" t="s">
-        <v>220</v>
+        <v>213</v>
       </c>
       <c r="F3" t="s">
         <v>69</v>
@@ -1522,10 +1501,10 @@
         <v>12</v>
       </c>
       <c r="C2" s="1" t="s">
+        <v>245</v>
+      </c>
+      <c r="D2" s="1" t="s">
         <v>252</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>259</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
@@ -1536,10 +1515,10 @@
         <v>13</v>
       </c>
       <c r="C3" s="1" t="s">
+        <v>245</v>
+      </c>
+      <c r="D3" s="1" t="s">
         <v>252</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>259</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
@@ -1550,10 +1529,10 @@
         <v>14</v>
       </c>
       <c r="C4" s="1" t="s">
+        <v>245</v>
+      </c>
+      <c r="D4" s="1" t="s">
         <v>252</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>259</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
@@ -1564,10 +1543,10 @@
         <v>15</v>
       </c>
       <c r="C5" s="1" t="s">
+        <v>245</v>
+      </c>
+      <c r="D5" s="1" t="s">
         <v>252</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>259</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
@@ -1578,10 +1557,10 @@
         <v>16</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>259</v>
+        <v>252</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>253</v>
+        <v>246</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
@@ -1592,10 +1571,10 @@
         <v>17</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>259</v>
+        <v>252</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>253</v>
+        <v>246</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">
@@ -1606,10 +1585,10 @@
         <v>18</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>259</v>
+        <v>252</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>253</v>
+        <v>246</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.2">
@@ -1620,10 +1599,10 @@
         <v>19</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>259</v>
+        <v>252</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>253</v>
+        <v>246</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.2">
@@ -1634,10 +1613,10 @@
         <v>20</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>259</v>
+        <v>252</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>253</v>
+        <v>246</v>
       </c>
     </row>
   </sheetData>
@@ -1663,7 +1642,7 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>222</v>
+        <v>215</v>
       </c>
       <c r="B2">
         <v>1</v>
@@ -1671,7 +1650,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>223</v>
+        <v>216</v>
       </c>
       <c r="B3">
         <v>2</v>
@@ -1679,7 +1658,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>224</v>
+        <v>217</v>
       </c>
       <c r="B4">
         <v>3</v>
@@ -1687,7 +1666,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>225</v>
+        <v>218</v>
       </c>
       <c r="B5">
         <v>4</v>
@@ -1695,7 +1674,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="B6">
         <v>5</v>
@@ -1703,7 +1682,7 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>227</v>
+        <v>220</v>
       </c>
       <c r="B7">
         <v>6</v>
@@ -1711,7 +1690,7 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>228</v>
+        <v>221</v>
       </c>
       <c r="B8">
         <v>7</v>
@@ -1719,7 +1698,7 @@
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>229</v>
+        <v>222</v>
       </c>
       <c r="B9">
         <v>8</v>
@@ -1727,7 +1706,7 @@
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>230</v>
+        <v>223</v>
       </c>
       <c r="B10">
         <v>9</v>
@@ -1735,7 +1714,7 @@
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>231</v>
+        <v>224</v>
       </c>
       <c r="B11">
         <v>10</v>
@@ -1743,7 +1722,7 @@
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>232</v>
+        <v>225</v>
       </c>
       <c r="B12">
         <v>11</v>
@@ -1751,7 +1730,7 @@
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>233</v>
+        <v>226</v>
       </c>
       <c r="B13">
         <v>12</v>
@@ -1759,7 +1738,7 @@
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>234</v>
+        <v>227</v>
       </c>
       <c r="B14">
         <v>13</v>
@@ -1767,7 +1746,7 @@
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>235</v>
+        <v>228</v>
       </c>
       <c r="B15">
         <v>14</v>
@@ -1775,7 +1754,7 @@
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>236</v>
+        <v>229</v>
       </c>
       <c r="B16">
         <v>15</v>
@@ -1783,7 +1762,7 @@
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>237</v>
+        <v>230</v>
       </c>
       <c r="B17">
         <v>16</v>
@@ -1791,7 +1770,7 @@
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>238</v>
+        <v>231</v>
       </c>
       <c r="B18">
         <v>17</v>
@@ -1799,7 +1778,7 @@
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>239</v>
+        <v>232</v>
       </c>
       <c r="B19">
         <v>18</v>
@@ -1807,7 +1786,7 @@
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>240</v>
+        <v>233</v>
       </c>
       <c r="B20">
         <v>19</v>
@@ -1815,7 +1794,7 @@
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>241</v>
+        <v>234</v>
       </c>
       <c r="B21">
         <v>20</v>
@@ -1823,7 +1802,7 @@
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>242</v>
+        <v>235</v>
       </c>
       <c r="B22">
         <v>21</v>
@@ -1831,7 +1810,7 @@
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>243</v>
+        <v>236</v>
       </c>
       <c r="B23">
         <v>22</v>
@@ -1839,7 +1818,7 @@
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>244</v>
+        <v>237</v>
       </c>
       <c r="B24">
         <v>23</v>
@@ -1847,7 +1826,7 @@
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>245</v>
+        <v>238</v>
       </c>
       <c r="B25">
         <v>24</v>
@@ -1855,7 +1834,7 @@
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>246</v>
+        <v>239</v>
       </c>
       <c r="B26">
         <v>25</v>
@@ -1863,7 +1842,7 @@
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>247</v>
+        <v>240</v>
       </c>
       <c r="B27">
         <v>26</v>
@@ -1871,7 +1850,7 @@
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>248</v>
+        <v>241</v>
       </c>
       <c r="B28">
         <v>27</v>
@@ -1879,7 +1858,7 @@
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>249</v>
+        <v>242</v>
       </c>
       <c r="B29">
         <v>28</v>
@@ -1946,7 +1925,7 @@
         <v>27</v>
       </c>
       <c r="B3">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="C3" t="s">
         <v>29</v>
@@ -2023,62 +2002,62 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="B7">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="C7" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D7" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="E7" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="F7" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B8">
         <v>7</v>
       </c>
       <c r="C8" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D8" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E8" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="F8" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="B9">
         <v>8</v>
       </c>
       <c r="C9" t="s">
-        <v>35</v>
+        <v>157</v>
       </c>
       <c r="D9" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E9" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="F9" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
@@ -2314,7 +2293,7 @@
         <v>96</v>
       </c>
       <c r="F7" t="s">
-        <v>254</v>
+        <v>247</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
@@ -2334,7 +2313,7 @@
         <v>97</v>
       </c>
       <c r="F8" t="s">
-        <v>255</v>
+        <v>248</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
@@ -2596,6 +2575,222 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
+  <dimension ref="A1:F10"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="2" width="12.6640625" customWidth="1"/>
+    <col min="3" max="3" width="100.6640625" customWidth="1"/>
+    <col min="4" max="5" width="20.6640625" customWidth="1"/>
+    <col min="6" max="6" width="60.6640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C1" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1" t="s">
+        <v>25</v>
+      </c>
+      <c r="E1" t="s">
+        <v>26</v>
+      </c>
+      <c r="F1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A2">
+        <v>14</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2" t="s">
+        <v>132</v>
+      </c>
+      <c r="D2" t="s">
+        <v>141</v>
+      </c>
+      <c r="E2" t="s">
+        <v>145</v>
+      </c>
+      <c r="F2" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A3">
+        <v>58</v>
+      </c>
+      <c r="B3">
+        <v>2</v>
+      </c>
+      <c r="C3" t="s">
+        <v>133</v>
+      </c>
+      <c r="D3" t="s">
+        <v>142</v>
+      </c>
+      <c r="E3" t="s">
+        <v>146</v>
+      </c>
+      <c r="F3" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A4">
+        <v>91</v>
+      </c>
+      <c r="B4">
+        <v>3</v>
+      </c>
+      <c r="C4" t="s">
+        <v>134</v>
+      </c>
+      <c r="D4" t="s">
+        <v>143</v>
+      </c>
+      <c r="E4" t="s">
+        <v>147</v>
+      </c>
+      <c r="F4" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A5">
+        <v>93</v>
+      </c>
+      <c r="B5">
+        <v>4</v>
+      </c>
+      <c r="C5" t="s">
+        <v>135</v>
+      </c>
+      <c r="D5" t="s">
+        <v>144</v>
+      </c>
+      <c r="E5" t="s">
+        <v>249</v>
+      </c>
+      <c r="F5" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A6">
+        <v>94</v>
+      </c>
+      <c r="B6">
+        <v>5</v>
+      </c>
+      <c r="C6" t="s">
+        <v>136</v>
+      </c>
+      <c r="D6" t="s">
+        <v>144</v>
+      </c>
+      <c r="E6" t="s">
+        <v>249</v>
+      </c>
+      <c r="F6" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A7">
+        <v>95</v>
+      </c>
+      <c r="B7">
+        <v>6</v>
+      </c>
+      <c r="C7" t="s">
+        <v>137</v>
+      </c>
+      <c r="D7" t="s">
+        <v>144</v>
+      </c>
+      <c r="E7" t="s">
+        <v>249</v>
+      </c>
+      <c r="F7" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A8">
+        <v>97</v>
+      </c>
+      <c r="B8">
+        <v>7</v>
+      </c>
+      <c r="C8" t="s">
+        <v>138</v>
+      </c>
+      <c r="D8" t="s">
+        <v>144</v>
+      </c>
+      <c r="E8" t="s">
+        <v>249</v>
+      </c>
+      <c r="F8" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A9">
+        <v>99</v>
+      </c>
+      <c r="B9">
+        <v>8</v>
+      </c>
+      <c r="C9" t="s">
+        <v>139</v>
+      </c>
+      <c r="D9" t="s">
+        <v>144</v>
+      </c>
+      <c r="E9" t="s">
+        <v>249</v>
+      </c>
+      <c r="F9" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A10">
+        <v>104</v>
+      </c>
+      <c r="B10">
+        <v>9</v>
+      </c>
+      <c r="C10" t="s">
+        <v>140</v>
+      </c>
+      <c r="D10" t="s">
+        <v>41</v>
+      </c>
+      <c r="E10" t="s">
+        <v>148</v>
+      </c>
+      <c r="F10" t="s">
+        <v>151</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
   <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
@@ -2627,258 +2822,22 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2">
-        <v>14</v>
-      </c>
-      <c r="B2">
-        <v>1</v>
-      </c>
-      <c r="C2" t="s">
-        <v>132</v>
-      </c>
-      <c r="D2" t="s">
-        <v>142</v>
-      </c>
-      <c r="E2" t="s">
-        <v>147</v>
-      </c>
-      <c r="F2" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A3">
-        <v>58</v>
-      </c>
-      <c r="B3">
-        <v>2</v>
-      </c>
-      <c r="C3" t="s">
-        <v>133</v>
-      </c>
-      <c r="D3" t="s">
-        <v>143</v>
-      </c>
-      <c r="E3" t="s">
-        <v>148</v>
-      </c>
-      <c r="F3" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A4">
-        <v>91</v>
-      </c>
-      <c r="B4">
-        <v>3</v>
-      </c>
-      <c r="C4" t="s">
-        <v>134</v>
-      </c>
-      <c r="D4" t="s">
-        <v>144</v>
-      </c>
-      <c r="E4" t="s">
-        <v>149</v>
-      </c>
-      <c r="F4" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A5">
-        <v>93</v>
-      </c>
-      <c r="B5">
-        <v>4</v>
-      </c>
-      <c r="C5" t="s">
-        <v>135</v>
-      </c>
-      <c r="D5" t="s">
-        <v>145</v>
-      </c>
-      <c r="E5" t="s">
-        <v>256</v>
-      </c>
-      <c r="F5" t="s">
-        <v>257</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A6">
-        <v>94</v>
-      </c>
-      <c r="B6">
-        <v>5</v>
-      </c>
-      <c r="C6" t="s">
-        <v>136</v>
-      </c>
-      <c r="D6" t="s">
-        <v>145</v>
-      </c>
-      <c r="E6" t="s">
-        <v>256</v>
-      </c>
-      <c r="F6" t="s">
-        <v>257</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A7">
-        <v>95</v>
-      </c>
-      <c r="B7">
-        <v>6</v>
-      </c>
-      <c r="C7" t="s">
-        <v>137</v>
-      </c>
-      <c r="D7" t="s">
-        <v>145</v>
-      </c>
-      <c r="E7" t="s">
-        <v>256</v>
-      </c>
-      <c r="F7" t="s">
-        <v>257</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A8">
-        <v>97</v>
-      </c>
-      <c r="B8">
-        <v>7</v>
-      </c>
-      <c r="C8" t="s">
-        <v>138</v>
-      </c>
-      <c r="D8" t="s">
-        <v>145</v>
-      </c>
-      <c r="E8" t="s">
-        <v>256</v>
-      </c>
-      <c r="F8" t="s">
-        <v>257</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A9">
-        <v>99</v>
-      </c>
-      <c r="B9">
-        <v>8</v>
-      </c>
-      <c r="C9" t="s">
-        <v>139</v>
-      </c>
-      <c r="D9" t="s">
-        <v>145</v>
-      </c>
-      <c r="E9" t="s">
-        <v>256</v>
-      </c>
-      <c r="F9" t="s">
-        <v>257</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A10">
-        <v>104</v>
-      </c>
-      <c r="B10">
-        <v>9</v>
-      </c>
-      <c r="C10" t="s">
-        <v>140</v>
-      </c>
-      <c r="D10" t="s">
-        <v>41</v>
-      </c>
-      <c r="E10" t="s">
-        <v>150</v>
-      </c>
-      <c r="F10" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A11">
-        <v>118</v>
-      </c>
-      <c r="B11">
-        <v>9</v>
-      </c>
-      <c r="C11" t="s">
-        <v>141</v>
-      </c>
-      <c r="D11" t="s">
-        <v>146</v>
-      </c>
-      <c r="E11" t="s">
-        <v>151</v>
-      </c>
-      <c r="F11" t="s">
-        <v>155</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
-  <dimension ref="A1:F12"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="2" width="12.6640625" customWidth="1"/>
-    <col min="3" max="3" width="100.6640625" customWidth="1"/>
-    <col min="4" max="5" width="20.6640625" customWidth="1"/>
-    <col min="6" max="6" width="60.6640625" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
-        <v>23</v>
-      </c>
-      <c r="B1" t="s">
-        <v>22</v>
-      </c>
-      <c r="C1" t="s">
-        <v>24</v>
-      </c>
-      <c r="D1" t="s">
-        <v>25</v>
-      </c>
-      <c r="E1" t="s">
-        <v>26</v>
-      </c>
-      <c r="F1" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A2">
         <v>30</v>
       </c>
       <c r="B2">
         <v>10</v>
       </c>
       <c r="C2" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="D2" t="s">
         <v>87</v>
       </c>
       <c r="E2" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="F2" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
@@ -2889,16 +2848,16 @@
         <v>11</v>
       </c>
       <c r="C3" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="D3" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="E3" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="F3" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
@@ -2909,16 +2868,16 @@
         <v>12</v>
       </c>
       <c r="C4" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="D4" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="E4" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="F4" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
@@ -2929,16 +2888,16 @@
         <v>13</v>
       </c>
       <c r="C5" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="D5" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="E5" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="F5" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
@@ -2949,136 +2908,116 @@
         <v>14</v>
       </c>
       <c r="C6" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="D6" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="E6" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="F6" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7">
-        <v>83</v>
+        <v>96</v>
       </c>
       <c r="B7">
         <v>15</v>
       </c>
       <c r="C7" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="D7" t="s">
-        <v>47</v>
+        <v>144</v>
       </c>
       <c r="E7" t="s">
-        <v>58</v>
+        <v>249</v>
       </c>
       <c r="F7" t="s">
-        <v>69</v>
+        <v>250</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8">
-        <v>96</v>
+        <v>105</v>
       </c>
       <c r="B8">
         <v>16</v>
       </c>
       <c r="C8" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="D8" t="s">
-        <v>145</v>
+        <v>167</v>
       </c>
       <c r="E8" t="s">
-        <v>256</v>
+        <v>175</v>
       </c>
       <c r="F8" t="s">
-        <v>257</v>
+        <v>184</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="B9">
         <v>17</v>
       </c>
       <c r="C9" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="D9" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="E9" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="F9" t="s">
-        <v>188</v>
+        <v>251</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10">
-        <v>108</v>
+        <v>120</v>
       </c>
       <c r="B10">
         <v>18</v>
       </c>
       <c r="C10" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="D10" t="s">
-        <v>172</v>
+        <v>113</v>
       </c>
       <c r="E10" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="F10" t="s">
-        <v>258</v>
+        <v>185</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11">
-        <v>120</v>
+        <v>136</v>
       </c>
       <c r="B11">
         <v>19</v>
       </c>
       <c r="C11" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="D11" t="s">
-        <v>113</v>
+        <v>169</v>
       </c>
       <c r="E11" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="F11" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A12">
-        <v>136</v>
-      </c>
-      <c r="B12">
-        <v>19</v>
-      </c>
-      <c r="C12" t="s">
-        <v>166</v>
-      </c>
-      <c r="D12" t="s">
-        <v>173</v>
-      </c>
-      <c r="E12" t="s">
-        <v>182</v>
-      </c>
-      <c r="F12" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
     </row>
   </sheetData>

</xml_diff>